<commit_message>
no longer using namespace std
</commit_message>
<xml_diff>
--- a/src/square45-90_sobel_exp.bin.hough.top.xlsx
+++ b/src/square45-90_sobel_exp.bin.hough.top.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,23 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kushn\Dropbox\software\projects\cv\cv-workbench\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D74D721-0708-474A-8141-EA2D424744E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC27E22-D902-411A-B226-E85380523345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="square45-90_sobel_exp.bin.hough" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'square45-90_sobel_exp.bin.hough'!$A$1:$X$7</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -549,18 +548,11 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF66FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF00FF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -879,7 +871,10 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:X7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1405,7 +1400,8 @@
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
+  <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="57" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>